<commit_message>
updated login logout system and fixed login history
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -399,7 +399,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>119500</v>
+        <v>134500</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -407,7 +407,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>45000</v>
+        <v>50000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified code for Business Analyzer project
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -399,7 +399,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>161050</v>
+        <v>183050</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -407,7 +407,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>68500</v>
+        <v>83500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>